<commit_message>
Forgot to apply stash
</commit_message>
<xml_diff>
--- a/documents/BoM.xlsx
+++ b/documents/BoM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aidan\sleep-wearable\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{02F71DF5-9252-4617-A502-8BA8CE2E43FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{476CE043-54E4-46F9-AF2D-A3BA08CB80D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19590" yWindow="-833" windowWidth="16200" windowHeight="9308" xr2:uid="{8E387801-223C-4F5F-AF87-1E267FE988A0}"/>
+    <workbookView xWindow="1402" yWindow="0" windowWidth="17738" windowHeight="12863" xr2:uid="{8E387801-223C-4F5F-AF87-1E267FE988A0}"/>
   </bookViews>
   <sheets>
     <sheet name="wearable" sheetId="1" r:id="rId1"/>
@@ -61,9 +61,6 @@
     <t>Estimated Tariff Price</t>
   </si>
   <si>
-    <t>Estimated Tariff Ext.</t>
-  </si>
-  <si>
     <t>BT1</t>
   </si>
   <si>
@@ -800,6 +797,9 @@
   </si>
   <si>
     <t>Analog to Digital Converters - ADC Analog to Digital Converters - ADC Low-Noise 4-Channel 24-Bit Analog-to-D A A 595-ADS1299-4PAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -945,7 +945,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1125,6 +1125,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1286,9 +1292,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1665,9 +1672,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDB4FCCF-8788-4C41-8DB3-AAD5ABBF3783}">
   <dimension ref="A1:N51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1708,36 +1715,36 @@
         <v>12</v>
       </c>
       <c r="N1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
         <v>16</v>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
       <c r="I2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1746,7 +1753,7 @@
         <v>0.1</v>
       </c>
       <c r="L2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M2" s="1">
         <v>1.6E-2</v>
@@ -1755,33 +1762,33 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>24</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
         <v>25</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>26</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>27</v>
       </c>
-      <c r="H3" t="s">
-        <v>28</v>
-      </c>
       <c r="I3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1790,7 +1797,7 @@
         <v>0.1</v>
       </c>
       <c r="L3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M3" s="1">
         <v>1.2999999999999999E-2</v>
@@ -1799,33 +1806,33 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
         <v>29</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
         <v>30</v>
       </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>31</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>32</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>33</v>
       </c>
-      <c r="H4" t="s">
-        <v>34</v>
-      </c>
       <c r="I4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -1834,7 +1841,7 @@
         <v>0.15</v>
       </c>
       <c r="L4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M4" s="1">
         <v>6.2E-2</v>
@@ -1843,33 +1850,33 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" t="s">
-        <v>36</v>
-      </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D5">
         <v>8</v>
       </c>
       <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
         <v>37</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>38</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>39</v>
       </c>
-      <c r="H5" t="s">
-        <v>40</v>
-      </c>
       <c r="I5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J5">
         <v>8</v>
@@ -1878,36 +1885,36 @@
         <v>0.76</v>
       </c>
       <c r="L5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
         <v>41</v>
       </c>
-      <c r="B6" t="s">
-        <v>42</v>
-      </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D6">
         <v>4</v>
       </c>
       <c r="E6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" t="s">
         <v>43</v>
       </c>
-      <c r="F6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="H6" t="s">
-        <v>45</v>
-      </c>
       <c r="I6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J6">
         <v>4</v>
@@ -1916,7 +1923,7 @@
         <v>0.12</v>
       </c>
       <c r="L6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M6" s="1">
         <v>1.4999999999999999E-2</v>
@@ -1925,33 +1932,33 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
         <v>46</v>
       </c>
-      <c r="B7" t="s">
-        <v>47</v>
-      </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D7">
         <v>5</v>
       </c>
       <c r="E7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" t="s">
         <v>48</v>
       </c>
-      <c r="F7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>49</v>
       </c>
-      <c r="H7" t="s">
-        <v>50</v>
-      </c>
       <c r="I7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J7">
         <v>5</v>
@@ -1960,7 +1967,7 @@
         <v>0.33</v>
       </c>
       <c r="L7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M7" s="1">
         <v>4.1000000000000002E-2</v>
@@ -1969,33 +1976,33 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
         <v>51</v>
       </c>
-      <c r="B8" t="s">
-        <v>52</v>
-      </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" t="s">
         <v>43</v>
       </c>
-      <c r="F8" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>44</v>
       </c>
-      <c r="H8" t="s">
-        <v>45</v>
-      </c>
       <c r="I8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -2004,7 +2011,7 @@
         <v>0.12</v>
       </c>
       <c r="L8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M8" s="1">
         <v>1.4999999999999999E-2</v>
@@ -2013,33 +2020,33 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" t="s">
         <v>53</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>54</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
         <v>55</v>
       </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>56</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>57</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>58</v>
       </c>
-      <c r="H9" t="s">
-        <v>59</v>
-      </c>
       <c r="I9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -2048,36 +2055,36 @@
         <v>0.99</v>
       </c>
       <c r="L9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
         <v>60</v>
       </c>
-      <c r="B10" t="s">
-        <v>61</v>
-      </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D10">
         <v>2</v>
       </c>
       <c r="E10" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" t="s">
         <v>62</v>
       </c>
-      <c r="F10" t="s">
-        <v>57</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>63</v>
       </c>
-      <c r="H10" t="s">
-        <v>64</v>
-      </c>
       <c r="I10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J10">
         <v>2</v>
@@ -2086,7 +2093,7 @@
         <v>0.32</v>
       </c>
       <c r="L10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M10" s="1">
         <v>3.2000000000000001E-2</v>
@@ -2095,33 +2102,33 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
         <v>65</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
         <v>66</v>
       </c>
-      <c r="C11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" t="s">
         <v>67</v>
       </c>
-      <c r="F11" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>68</v>
       </c>
-      <c r="H11" t="s">
-        <v>69</v>
-      </c>
       <c r="I11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -2130,36 +2137,36 @@
         <v>0.83</v>
       </c>
       <c r="L11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" t="s">
         <v>70</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
         <v>71</v>
       </c>
-      <c r="C12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" t="s">
         <v>72</v>
       </c>
-      <c r="F12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>73</v>
       </c>
-      <c r="H12" t="s">
-        <v>74</v>
-      </c>
       <c r="I12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -2168,7 +2175,7 @@
         <v>0.17</v>
       </c>
       <c r="L12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M12" s="1">
         <v>2.1000000000000001E-2</v>
@@ -2177,33 +2184,33 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" t="s">
         <v>75</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
         <v>76</v>
       </c>
-      <c r="C13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" t="s">
         <v>77</v>
       </c>
-      <c r="F13" t="s">
-        <v>32</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>78</v>
       </c>
-      <c r="H13" t="s">
-        <v>79</v>
-      </c>
       <c r="I13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -2212,36 +2219,36 @@
         <v>0.78</v>
       </c>
       <c r="L13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" t="s">
         <v>80</v>
       </c>
-      <c r="B14" t="s">
-        <v>81</v>
-      </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D14">
         <v>5</v>
       </c>
       <c r="E14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" t="s">
         <v>82</v>
       </c>
-      <c r="F14" t="s">
-        <v>26</v>
-      </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>83</v>
       </c>
-      <c r="H14" t="s">
-        <v>84</v>
-      </c>
       <c r="I14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J14">
         <v>5</v>
@@ -2250,7 +2257,7 @@
         <v>0.21</v>
       </c>
       <c r="L14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M14" s="1">
         <v>2.5999999999999999E-2</v>
@@ -2259,50 +2266,50 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" t="s">
         <v>85</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>86</v>
-      </c>
-      <c r="C15" t="s">
-        <v>87</v>
       </c>
       <c r="D15">
         <v>2</v>
       </c>
       <c r="E15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>89</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>90</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
         <v>91</v>
       </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>92</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>93</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>94</v>
       </c>
-      <c r="H16" t="s">
-        <v>95</v>
-      </c>
       <c r="I16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -2311,7 +2318,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="L16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M16" s="1">
         <v>2.4E-2</v>
@@ -2320,33 +2327,33 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" t="s">
         <v>96</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>97</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
         <v>98</v>
       </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>99</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>100</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>101</v>
       </c>
-      <c r="H17" t="s">
-        <v>102</v>
-      </c>
       <c r="I17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J17">
         <v>1</v>
@@ -2355,7 +2362,7 @@
         <v>0.69</v>
       </c>
       <c r="L17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M17" s="1">
         <v>0.38600000000000001</v>
@@ -2364,47 +2371,47 @@
         <v>0.39</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="s">
         <v>103</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>104</v>
-      </c>
-      <c r="C18" t="s">
-        <v>105</v>
       </c>
       <c r="D18">
         <v>5</v>
       </c>
       <c r="E18" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" t="s">
         <v>106</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>107</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="s">
         <v>108</v>
       </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>109</v>
       </c>
-      <c r="F19" t="s">
+      <c r="H19" t="s">
         <v>110</v>
       </c>
-      <c r="H19" t="s">
-        <v>111</v>
-      </c>
       <c r="I19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -2413,53 +2420,53 @@
         <v>1.95</v>
       </c>
       <c r="L19" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
+        <v>111</v>
+      </c>
+      <c r="B20" t="s">
         <v>112</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>113</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
         <v>114</v>
       </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
         <v>115</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>116</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" t="s">
         <v>117</v>
       </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>118</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>119</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>120</v>
       </c>
-      <c r="H21" t="s">
-        <v>121</v>
-      </c>
       <c r="I21" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J21">
         <v>1</v>
@@ -2468,7 +2475,7 @@
         <v>0.6</v>
       </c>
       <c r="L21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M21" s="1">
         <v>0.23799999999999999</v>
@@ -2477,33 +2484,33 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" t="s">
         <v>122</v>
       </c>
-      <c r="B22" t="s">
-        <v>123</v>
-      </c>
       <c r="C22" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
         <v>117</v>
       </c>
-      <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>118</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>119</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>120</v>
       </c>
-      <c r="H22" t="s">
-        <v>121</v>
-      </c>
       <c r="I22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J22">
         <v>1</v>
@@ -2512,7 +2519,7 @@
         <v>0.6</v>
       </c>
       <c r="L22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M22" s="1">
         <v>0.23799999999999999</v>
@@ -2521,50 +2528,50 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
+        <v>123</v>
+      </c>
+      <c r="B23" t="s">
         <v>124</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>125</v>
-      </c>
-      <c r="C23" t="s">
-        <v>126</v>
       </c>
       <c r="D23">
         <v>11</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>128</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" t="s">
         <v>129</v>
       </c>
-      <c r="C24" t="s">
-        <v>126</v>
-      </c>
-      <c r="D24">
-        <v>1</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
+        <v>31</v>
+      </c>
+      <c r="G24" t="s">
         <v>130</v>
       </c>
-      <c r="F24" t="s">
-        <v>32</v>
-      </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>131</v>
       </c>
-      <c r="H24" t="s">
-        <v>132</v>
-      </c>
       <c r="I24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J24">
         <v>1</v>
@@ -2573,7 +2580,7 @@
         <v>0.66</v>
       </c>
       <c r="L24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M24" s="1">
         <v>9.1999999999999998E-2</v>
@@ -2582,33 +2589,33 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" t="s">
         <v>133</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
+        <v>125</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25" t="s">
         <v>134</v>
       </c>
-      <c r="C25" t="s">
-        <v>126</v>
-      </c>
-      <c r="D25">
-        <v>1</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>135</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>136</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>137</v>
       </c>
-      <c r="H25" t="s">
-        <v>138</v>
-      </c>
       <c r="I25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J25">
         <v>1</v>
@@ -2617,53 +2624,53 @@
         <v>0.1</v>
       </c>
       <c r="L25" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B26">
         <v>330</v>
       </c>
       <c r="C26" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D26">
         <v>1</v>
       </c>
       <c r="E26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
         <v>140</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>141</v>
       </c>
       <c r="B27">
         <v>820</v>
       </c>
       <c r="C27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D27">
         <v>1</v>
       </c>
       <c r="E27" t="s">
+        <v>141</v>
+      </c>
+      <c r="F27" t="s">
         <v>142</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>143</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>144</v>
       </c>
-      <c r="H27" t="s">
-        <v>145</v>
-      </c>
       <c r="I27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J27">
         <v>1</v>
@@ -2672,36 +2679,36 @@
         <v>0.1</v>
       </c>
       <c r="L27" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
+        <v>145</v>
+      </c>
+      <c r="B28" t="s">
         <v>146</v>
       </c>
-      <c r="B28" t="s">
-        <v>147</v>
-      </c>
       <c r="C28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D28">
         <v>3</v>
       </c>
       <c r="E28" t="s">
+        <v>147</v>
+      </c>
+      <c r="F28" t="s">
+        <v>142</v>
+      </c>
+      <c r="G28" t="s">
+        <v>143</v>
+      </c>
+      <c r="H28" t="s">
         <v>148</v>
       </c>
-      <c r="F28" t="s">
-        <v>143</v>
-      </c>
-      <c r="G28" t="s">
-        <v>144</v>
-      </c>
-      <c r="H28" t="s">
-        <v>149</v>
-      </c>
       <c r="I28" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J28">
         <v>3</v>
@@ -2710,36 +2717,36 @@
         <v>0.13</v>
       </c>
       <c r="L28" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
+        <v>149</v>
+      </c>
+      <c r="B29" t="s">
         <v>150</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
+        <v>125</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29" t="s">
         <v>151</v>
       </c>
-      <c r="C29" t="s">
-        <v>126</v>
-      </c>
-      <c r="D29">
-        <v>1</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>152</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>153</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>154</v>
       </c>
-      <c r="H29" t="s">
-        <v>155</v>
-      </c>
       <c r="I29" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J29">
         <v>1</v>
@@ -2748,7 +2755,7 @@
         <v>0.12</v>
       </c>
       <c r="L29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M29" s="1">
         <v>1.7000000000000001E-2</v>
@@ -2757,33 +2764,33 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
+        <v>155</v>
+      </c>
+      <c r="B30" t="s">
         <v>156</v>
       </c>
-      <c r="B30" t="s">
-        <v>157</v>
-      </c>
       <c r="C30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D30">
         <v>2</v>
       </c>
       <c r="E30" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" t="s">
         <v>158</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>159</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>160</v>
       </c>
-      <c r="H30" t="s">
-        <v>161</v>
-      </c>
       <c r="I30" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J30">
         <v>2</v>
@@ -2792,7 +2799,7 @@
         <v>0.2</v>
       </c>
       <c r="L30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M30" s="1">
         <v>0.04</v>
@@ -2801,33 +2808,33 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B31">
         <v>499</v>
       </c>
       <c r="C31" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D31">
         <v>1</v>
       </c>
       <c r="E31" t="s">
+        <v>162</v>
+      </c>
+      <c r="F31" t="s">
+        <v>152</v>
+      </c>
+      <c r="G31" t="s">
         <v>163</v>
       </c>
-      <c r="F31" t="s">
-        <v>153</v>
-      </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>164</v>
       </c>
-      <c r="H31" t="s">
-        <v>165</v>
-      </c>
       <c r="I31" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J31">
         <v>1</v>
@@ -2836,7 +2843,7 @@
         <v>1.25</v>
       </c>
       <c r="L31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M31" s="1">
         <v>0.17499999999999999</v>
@@ -2845,33 +2852,33 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
+        <v>165</v>
+      </c>
+      <c r="B32" t="s">
         <v>166</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
+        <v>125</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32" t="s">
         <v>167</v>
       </c>
-      <c r="C32" t="s">
-        <v>126</v>
-      </c>
-      <c r="D32">
-        <v>1</v>
-      </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
+        <v>31</v>
+      </c>
+      <c r="G32" t="s">
         <v>168</v>
       </c>
-      <c r="F32" t="s">
-        <v>32</v>
-      </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>169</v>
       </c>
-      <c r="H32" t="s">
-        <v>170</v>
-      </c>
       <c r="I32" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J32">
         <v>1</v>
@@ -2880,7 +2887,7 @@
         <v>0.82</v>
       </c>
       <c r="L32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M32" s="1">
         <v>0.115</v>
@@ -2889,33 +2896,33 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
+        <v>170</v>
+      </c>
+      <c r="B33" t="s">
         <v>171</v>
       </c>
-      <c r="B33" t="s">
-        <v>172</v>
-      </c>
       <c r="C33" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D33">
         <v>2</v>
       </c>
       <c r="E33" t="s">
+        <v>172</v>
+      </c>
+      <c r="F33" t="s">
+        <v>31</v>
+      </c>
+      <c r="G33" t="s">
         <v>173</v>
       </c>
-      <c r="F33" t="s">
-        <v>32</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>174</v>
       </c>
-      <c r="H33" t="s">
-        <v>175</v>
-      </c>
       <c r="I33" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J33">
         <v>2</v>
@@ -2924,36 +2931,36 @@
         <v>0.83</v>
       </c>
       <c r="L33" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
+        <v>175</v>
+      </c>
+      <c r="B34" t="s">
         <v>176</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
+        <v>125</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34" t="s">
         <v>177</v>
       </c>
-      <c r="C34" t="s">
-        <v>126</v>
-      </c>
-      <c r="D34">
-        <v>1</v>
-      </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
+        <v>135</v>
+      </c>
+      <c r="G34" t="s">
         <v>178</v>
       </c>
-      <c r="F34" t="s">
-        <v>136</v>
-      </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>179</v>
       </c>
-      <c r="H34" t="s">
-        <v>180</v>
-      </c>
       <c r="I34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J34">
         <v>1</v>
@@ -2962,121 +2969,121 @@
         <v>0.68</v>
       </c>
       <c r="L34" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
+        <v>180</v>
+      </c>
+      <c r="B35" t="s">
         <v>181</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>182</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
         <v>183</v>
       </c>
-      <c r="D35">
-        <v>1</v>
-      </c>
-      <c r="E35" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
         <v>184</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>185</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
         <v>186</v>
       </c>
-      <c r="D36">
-        <v>1</v>
-      </c>
-      <c r="E36" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="B37" t="s">
         <v>187</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
+        <v>185</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
         <v>188</v>
       </c>
-      <c r="C37" t="s">
-        <v>186</v>
-      </c>
-      <c r="D37">
-        <v>1</v>
-      </c>
-      <c r="E37" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="B38" t="s">
         <v>189</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>190</v>
-      </c>
-      <c r="C38" t="s">
-        <v>191</v>
       </c>
       <c r="D38">
         <v>13</v>
       </c>
       <c r="E38" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
+        <v>191</v>
+      </c>
+      <c r="B39" t="s">
         <v>192</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>193</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39" t="s">
         <v>194</v>
       </c>
-      <c r="D39">
-        <v>1</v>
-      </c>
-      <c r="E39" t="s">
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="B40" t="s">
         <v>196</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>197</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40" t="s">
         <v>198</v>
       </c>
-      <c r="D40">
-        <v>1</v>
-      </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
+        <v>99</v>
+      </c>
+      <c r="G40" t="s">
+        <v>100</v>
+      </c>
+      <c r="H40" t="s">
         <v>199</v>
       </c>
-      <c r="F40" t="s">
-        <v>100</v>
-      </c>
-      <c r="G40" t="s">
-        <v>101</v>
-      </c>
-      <c r="H40" t="s">
-        <v>200</v>
-      </c>
       <c r="I40" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J40">
         <v>1</v>
@@ -3085,7 +3092,7 @@
         <v>0.49</v>
       </c>
       <c r="L40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M40" s="1">
         <v>0.27400000000000002</v>
@@ -3094,33 +3101,33 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
+        <v>200</v>
+      </c>
+      <c r="B41" t="s">
         <v>201</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" t="s">
         <v>202</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41" t="s">
         <v>203</v>
       </c>
-      <c r="D41">
-        <v>1</v>
-      </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>204</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>205</v>
       </c>
-      <c r="G41" t="s">
+      <c r="H41" t="s">
         <v>206</v>
       </c>
-      <c r="H41" t="s">
-        <v>207</v>
-      </c>
       <c r="I41" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J41">
         <v>1</v>
@@ -3129,33 +3136,33 @@
         <v>13.4</v>
       </c>
       <c r="L41" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
+        <v>207</v>
+      </c>
+      <c r="B42" t="s">
         <v>208</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>209</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42" t="s">
         <v>210</v>
       </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
         <v>211</v>
       </c>
-      <c r="F42" t="s">
+      <c r="H42" t="s">
         <v>212</v>
       </c>
-      <c r="H42" t="s">
-        <v>213</v>
-      </c>
       <c r="I42" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="J42">
         <v>1</v>
@@ -3164,36 +3171,36 @@
         <v>1.53</v>
       </c>
       <c r="L42" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
+        <v>213</v>
+      </c>
+      <c r="B43" t="s">
         <v>214</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>215</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="E43" t="s">
         <v>216</v>
       </c>
-      <c r="D43">
-        <v>1</v>
-      </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
         <v>217</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>218</v>
       </c>
-      <c r="G43" t="s">
+      <c r="H43" t="s">
         <v>219</v>
       </c>
-      <c r="H43" t="s">
+      <c r="I43" t="s">
         <v>220</v>
-      </c>
-      <c r="I43" t="s">
-        <v>221</v>
       </c>
       <c r="J43">
         <v>1</v>
@@ -3202,36 +3209,36 @@
         <v>9.24</v>
       </c>
       <c r="L43" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
+        <v>221</v>
+      </c>
+      <c r="B44" t="s">
         <v>222</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>223</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44">
+        <v>1</v>
+      </c>
+      <c r="E44" t="s">
         <v>224</v>
       </c>
-      <c r="D44">
-        <v>1</v>
-      </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
+        <v>99</v>
+      </c>
+      <c r="G44" t="s">
         <v>225</v>
       </c>
-      <c r="F44" t="s">
-        <v>100</v>
-      </c>
-      <c r="G44" t="s">
+      <c r="H44" t="s">
         <v>226</v>
       </c>
-      <c r="H44" t="s">
-        <v>227</v>
-      </c>
       <c r="I44" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J44">
         <v>1</v>
@@ -3240,7 +3247,7 @@
         <v>1.25</v>
       </c>
       <c r="L44" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M44" s="1">
         <v>0.7</v>
@@ -3249,33 +3256,33 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
+        <v>227</v>
+      </c>
+      <c r="B45" t="s">
         <v>228</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>229</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45" t="s">
         <v>230</v>
       </c>
-      <c r="D45">
-        <v>1</v>
-      </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>231</v>
       </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
         <v>232</v>
       </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>233</v>
       </c>
-      <c r="H45" t="s">
-        <v>234</v>
-      </c>
       <c r="I45" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J45">
         <v>1</v>
@@ -3284,36 +3291,36 @@
         <v>4.25</v>
       </c>
       <c r="L45" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
+        <v>234</v>
+      </c>
+      <c r="B46" t="s">
         <v>235</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>236</v>
-      </c>
-      <c r="C46" t="s">
-        <v>237</v>
       </c>
       <c r="D46">
         <v>2</v>
       </c>
       <c r="E46" t="s">
+        <v>237</v>
+      </c>
+      <c r="F46" t="s">
         <v>238</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>239</v>
       </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>240</v>
       </c>
-      <c r="H46" t="s">
+      <c r="I46" t="s">
         <v>241</v>
-      </c>
-      <c r="I46" t="s">
-        <v>242</v>
       </c>
       <c r="J46">
         <v>2</v>
@@ -3322,27 +3329,27 @@
         <v>1.64</v>
       </c>
       <c r="L46" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.45">
       <c r="D47">
         <v>1</v>
       </c>
       <c r="E47" t="s">
+        <v>242</v>
+      </c>
+      <c r="F47" t="s">
         <v>243</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>244</v>
       </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>245</v>
       </c>
-      <c r="H47" t="s">
-        <v>246</v>
-      </c>
       <c r="I47" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J47">
         <v>1</v>
@@ -3351,7 +3358,7 @@
         <v>0.23</v>
       </c>
       <c r="L47" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M47" s="1">
         <v>3.6999999999999998E-2</v>
@@ -3360,24 +3367,24 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.45">
       <c r="D48">
         <v>1</v>
       </c>
       <c r="E48" t="s">
+        <v>246</v>
+      </c>
+      <c r="F48" t="s">
         <v>247</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>248</v>
       </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>249</v>
       </c>
-      <c r="H48" t="s">
-        <v>250</v>
-      </c>
       <c r="I48" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J48">
         <v>1</v>
@@ -3386,7 +3393,7 @@
         <v>0.45</v>
       </c>
       <c r="L48" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M48" s="1">
         <v>7.1999999999999995E-2</v>
@@ -3395,21 +3402,21 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="49" spans="4:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:14" x14ac:dyDescent="0.45">
       <c r="D49">
         <v>1</v>
       </c>
       <c r="E49" t="s">
+        <v>250</v>
+      </c>
+      <c r="F49" t="s">
+        <v>109</v>
+      </c>
+      <c r="H49" t="s">
         <v>251</v>
       </c>
-      <c r="F49" t="s">
-        <v>110</v>
-      </c>
-      <c r="H49" t="s">
-        <v>252</v>
-      </c>
       <c r="I49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J49">
         <v>1</v>
@@ -3418,27 +3425,27 @@
         <v>3.5</v>
       </c>
       <c r="L49" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="50" spans="4:14" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="50" spans="4:14" x14ac:dyDescent="0.45">
       <c r="D50">
         <v>1</v>
       </c>
       <c r="E50" t="s">
+        <v>252</v>
+      </c>
+      <c r="F50" t="s">
         <v>253</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
         <v>254</v>
       </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>255</v>
       </c>
-      <c r="H50" t="s">
-        <v>256</v>
-      </c>
       <c r="I50" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="J50">
         <v>1</v>
@@ -3447,7 +3454,7 @@
         <v>5.3</v>
       </c>
       <c r="L50" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M50" s="1">
         <v>0.63600000000000001</v>
@@ -3456,24 +3463,24 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="51" spans="4:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="4:14" x14ac:dyDescent="0.45">
       <c r="D51">
         <v>1</v>
       </c>
       <c r="E51" t="s">
+        <v>256</v>
+      </c>
+      <c r="F51" t="s">
+        <v>99</v>
+      </c>
+      <c r="G51" t="s">
         <v>257</v>
       </c>
-      <c r="F51" t="s">
-        <v>100</v>
-      </c>
-      <c r="G51" t="s">
+      <c r="H51" t="s">
         <v>258</v>
       </c>
-      <c r="H51" t="s">
-        <v>259</v>
-      </c>
       <c r="I51" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J51">
         <v>1</v>
@@ -3482,7 +3489,7 @@
         <v>43.65</v>
       </c>
       <c r="L51" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>